<commit_message>
Direct Write Excel for CUTTER GRINDING-01 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTER GRINDING-01.xlsx
+++ b/FM-MN-07_CUTTER GRINDING-01.xlsx
@@ -1740,7 +1740,11 @@
       <c r="E6" s="13" t="inlineStr"/>
       <c r="F6" s="13" t="inlineStr"/>
       <c r="G6" s="13" t="inlineStr"/>
-      <c r="H6" s="13" t="inlineStr"/>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="13" t="inlineStr"/>
       <c r="J6" s="13" t="inlineStr"/>
       <c r="K6" s="13" t="inlineStr"/>
@@ -1781,7 +1785,11 @@
       <c r="E7" s="13" t="inlineStr"/>
       <c r="F7" s="13" t="inlineStr"/>
       <c r="G7" s="13" t="inlineStr"/>
-      <c r="H7" s="13" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="13" t="inlineStr"/>
       <c r="J7" s="13" t="inlineStr"/>
       <c r="K7" s="13" t="inlineStr"/>
@@ -1822,7 +1830,11 @@
       <c r="E8" s="13" t="inlineStr"/>
       <c r="F8" s="13" t="inlineStr"/>
       <c r="G8" s="13" t="inlineStr"/>
-      <c r="H8" s="13" t="inlineStr"/>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="13" t="inlineStr"/>
       <c r="J8" s="13" t="inlineStr"/>
       <c r="K8" s="13" t="inlineStr"/>
@@ -1863,7 +1875,11 @@
       <c r="E9" s="13" t="inlineStr"/>
       <c r="F9" s="13" t="inlineStr"/>
       <c r="G9" s="13" t="inlineStr"/>
-      <c r="H9" s="13" t="inlineStr"/>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="13" t="inlineStr"/>
       <c r="J9" s="13" t="inlineStr"/>
       <c r="K9" s="13" t="inlineStr"/>
@@ -1904,7 +1920,11 @@
       <c r="E10" s="13" t="inlineStr"/>
       <c r="F10" s="13" t="inlineStr"/>
       <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="13" t="inlineStr"/>
       <c r="J10" s="13" t="inlineStr"/>
       <c r="K10" s="13" t="inlineStr"/>
@@ -2009,7 +2029,11 @@
       <c r="E13" s="25" t="inlineStr"/>
       <c r="F13" s="25" t="inlineStr"/>
       <c r="G13" s="25" t="inlineStr"/>
-      <c r="H13" s="25" t="inlineStr"/>
+      <c r="H13" s="33" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="I13" s="25" t="inlineStr"/>
       <c r="J13" s="25" t="inlineStr"/>
       <c r="K13" s="25" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CUTTER GRINDING-01 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTER GRINDING-01.xlsx
+++ b/FM-MN-07_CUTTER GRINDING-01.xlsx
@@ -1745,7 +1745,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="13" t="inlineStr"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="13" t="inlineStr"/>
       <c r="K6" s="13" t="inlineStr"/>
       <c r="L6" s="13" t="inlineStr"/>
@@ -1790,7 +1794,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="13" t="inlineStr"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="13" t="inlineStr"/>
       <c r="K7" s="13" t="inlineStr"/>
       <c r="L7" s="13" t="inlineStr"/>
@@ -1835,7 +1843,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="13" t="inlineStr"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="13" t="inlineStr"/>
       <c r="K8" s="13" t="inlineStr"/>
       <c r="L8" s="13" t="inlineStr"/>
@@ -1880,7 +1892,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="13" t="inlineStr"/>
       <c r="K9" s="13" t="inlineStr"/>
       <c r="L9" s="13" t="inlineStr"/>
@@ -1925,7 +1941,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="13" t="inlineStr"/>
       <c r="K10" s="13" t="inlineStr"/>
       <c r="L10" s="13" t="inlineStr"/>
@@ -2034,7 +2054,11 @@
           <t>ณัช วิกรัยเจริญ</t>
         </is>
       </c>
-      <c r="I13" s="25" t="inlineStr"/>
+      <c r="I13" s="33" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="J13" s="25" t="inlineStr"/>
       <c r="K13" s="25" t="inlineStr"/>
       <c r="L13" s="25" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CUTTER GRINDING-01 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTER GRINDING-01.xlsx
+++ b/FM-MN-07_CUTTER GRINDING-01.xlsx
@@ -1750,7 +1750,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="13" t="inlineStr"/>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="13" t="inlineStr"/>
       <c r="L6" s="13" t="inlineStr"/>
       <c r="M6" s="13" t="inlineStr"/>
@@ -1799,7 +1803,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="13" t="inlineStr"/>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="13" t="inlineStr"/>
       <c r="L7" s="13" t="inlineStr"/>
       <c r="M7" s="13" t="inlineStr"/>
@@ -1848,7 +1856,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="13" t="inlineStr"/>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="13" t="inlineStr"/>
       <c r="L8" s="13" t="inlineStr"/>
       <c r="M8" s="13" t="inlineStr"/>
@@ -1897,7 +1909,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="13" t="inlineStr"/>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="13" t="inlineStr"/>
       <c r="L9" s="13" t="inlineStr"/>
       <c r="M9" s="13" t="inlineStr"/>
@@ -1946,7 +1962,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr"/>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="13" t="inlineStr"/>
       <c r="L10" s="13" t="inlineStr"/>
       <c r="M10" s="13" t="inlineStr"/>
@@ -2059,7 +2079,11 @@
           <t>ณัช วิกรัยเจริญ</t>
         </is>
       </c>
-      <c r="J13" s="25" t="inlineStr"/>
+      <c r="J13" s="33" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="K13" s="25" t="inlineStr"/>
       <c r="L13" s="25" t="inlineStr"/>
       <c r="M13" s="25" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CUTTER GRINDING-01 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTER GRINDING-01.xlsx
+++ b/FM-MN-07_CUTTER GRINDING-01.xlsx
@@ -1756,7 +1756,11 @@
         </is>
       </c>
       <c r="K6" s="13" t="inlineStr"/>
-      <c r="L6" s="13" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="13" t="inlineStr"/>
       <c r="N6" s="13" t="inlineStr"/>
       <c r="O6" s="13" t="inlineStr"/>
@@ -1809,7 +1813,11 @@
         </is>
       </c>
       <c r="K7" s="13" t="inlineStr"/>
-      <c r="L7" s="13" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="13" t="inlineStr"/>
       <c r="N7" s="13" t="inlineStr"/>
       <c r="O7" s="13" t="inlineStr"/>
@@ -1862,7 +1870,11 @@
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr"/>
-      <c r="L8" s="13" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="13" t="inlineStr"/>
       <c r="N8" s="13" t="inlineStr"/>
       <c r="O8" s="13" t="inlineStr"/>
@@ -1915,7 +1927,11 @@
         </is>
       </c>
       <c r="K9" s="13" t="inlineStr"/>
-      <c r="L9" s="13" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="13" t="inlineStr"/>
       <c r="N9" s="13" t="inlineStr"/>
       <c r="O9" s="13" t="inlineStr"/>
@@ -1968,7 +1984,11 @@
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr"/>
-      <c r="L10" s="13" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="13" t="inlineStr"/>
       <c r="N10" s="13" t="inlineStr"/>
       <c r="O10" s="13" t="inlineStr"/>
@@ -2085,7 +2105,11 @@
         </is>
       </c>
       <c r="K13" s="25" t="inlineStr"/>
-      <c r="L13" s="25" t="inlineStr"/>
+      <c r="L13" s="33" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="M13" s="25" t="inlineStr"/>
       <c r="N13" s="25" t="inlineStr"/>
       <c r="O13" s="25" t="inlineStr"/>

</xml_diff>